<commit_message>
chore: update schedules 2026-08-14
</commit_message>
<xml_diff>
--- a/output/esl_schedules_latest.xlsx
+++ b/output/esl_schedules_latest.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J95"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -524,7 +524,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
+          <t>16-Aug-2026</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>06-Sep-2026</t>
+          <t>05-Sep-2026</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -572,7 +572,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>03-Sep-2026</t>
+          <t>30-Aug-2026</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -791,28 +791,28 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ESL NHAVA SHEVA / 026D4</t>
+          <t>ESL NHAVA SHEVA / 026E1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>19 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>16-Sep-2026</t>
+          <t>03-Sep-2026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -839,28 +839,28 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ESL NINGBO / 026E3</t>
+          <t>ESL TBN01 / 026D4</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>19 days</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>19-Sep-2026</t>
+          <t>16-Sep-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -887,12 +887,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM / 026E1</t>
+          <t>ESL NINGBO / 026E2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -902,13 +902,13 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>20 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>17-Sep-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -935,28 +935,28 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>WIDE ALPHA / 026D6</t>
+          <t>KMTC DAMMAM / 026E3</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>19 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -983,28 +983,28 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>KMTC COLOMBO / 026E2</t>
+          <t>ESL TBN01 / 026E4</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>19 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>04-Oct-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1031,28 +1031,28 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN / 026E5</t>
+          <t>WIDE ALPHA / 026D6</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>19 days</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>05-Oct-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1079,28 +1079,28 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM / 026E6</t>
+          <t>KMTC COLOMBO / 026E2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>19 days</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>08-Oct-2026</t>
+          <t>03-Oct-2026</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1127,28 +1127,28 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ESL BUSAN / 026E3</t>
+          <t>BHUDTHI BHUM / 026E6</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>19 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>18-Oct-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1175,28 +1175,28 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>PHOEBE / 026E8</t>
+          <t>ESL TBN1 / 026E3</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>21 days</t>
+          <t>19 days</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1228,7 +1228,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ESL EFFICIENCY / 026E5</t>
+          <t>ESL BUSAN / 026E5</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1244,7 +1244,7 @@
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
+          <t>16-Aug-2026</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>06-Sep-2026</t>
+          <t>05-Sep-2026</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1573,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>03-Sep-2026</t>
+          <t>30-Aug-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1588,7 +1588,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>026D4</t>
+          <t>026E1</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1598,17 +1598,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1625,22 +1625,22 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>16-Sep-2026</t>
+          <t>03-Sep-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>026E3</t>
+          <t>026D4</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1650,17 +1650,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>19-Sep-2026</t>
+          <t>16-Sep-2026</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1687,12 +1687,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>026E1</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1702,17 +1702,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1729,22 +1729,22 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>17-Sep-2026</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>WIDE ALPHA</t>
+          <t>KMTC DAMMAM</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>026D6</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1754,17 +1754,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>13-Oct-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1781,22 +1781,22 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>KMTC COLOMBO</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>026E2</t>
+          <t>026E4</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1806,17 +1806,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1833,22 +1833,22 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>04-Oct-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>ESL KHOR FAKKAN</t>
+          <t>WIDE ALPHA</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>026E5</t>
+          <t>026D6</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1858,17 +1858,17 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>13-Oct-2026</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1885,22 +1885,22 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>05-Oct-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>KMTC COLOMBO</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1910,17 +1910,17 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1937,22 +1937,22 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>08-Oct-2026</t>
+          <t>03-Oct-2026</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ECMX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>ESL BUSAN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>026E3</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1962,17 +1962,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>27-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -1989,22 +1989,22 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>18-Oct-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL TBN1</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>026E8</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2014,17 +2014,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>27-Oct-2026</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>ESL EFFICIENCY</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2076,7 +2076,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:53 UTC</t>
         </is>
       </c>
     </row>
@@ -2093,38 +2093,38 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>09-Aug-2026</t>
+          <t>12-Aug-2026</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>19-Aug-2026</t>
+          <t>05-Sep-2026</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>EVER LIVING / 02630</t>
+          <t>BHUDTHI BHUM / 026D7</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>24 days</t>
         </is>
       </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2136,43 +2136,43 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>QINGDAO</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>16-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>PORT KLANG</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>20-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>05-Sep-2026</t>
+          <t>25-Aug-2026</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>ESL OMAN / 02633</t>
+          <t>ITAL USODIMARE / 02632</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>9 days</t>
         </is>
       </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2184,12 +2184,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>12-Aug-2026</t>
+          <t>01-Sep-2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2199,28 +2199,28 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>06-Sep-2026</t>
+          <t>12-Sep-2026</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM / 026D7</t>
+          <t>ESL BUSAN / 02634</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>25 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2237,38 +2237,38 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>16-Aug-2026</t>
+          <t>21-Aug-2026</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>25-Aug-2026</t>
+          <t>13-Sep-2026</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>ITAL USODIMARE / 02632</t>
+          <t>PHOEBE / 026D9</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>9 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2280,43 +2280,43 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>QINGDAO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>22-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>PORT KLANG</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>01-Sep-2026</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>12-Sep-2026</t>
-        </is>
-      </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>ESL BUSAN / 02634</t>
+          <t>EVER STEADY / 02633</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>11 days</t>
+          <t>10 days</t>
         </is>
       </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>21-Aug-2026</t>
+          <t>28-Aug-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2343,12 +2343,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>13-Sep-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>PHOEBE / 026D9</t>
+          <t>ESL NHAVA SHEVA / 026E1</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2364,7 +2364,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>22-Aug-2026</t>
+          <t>07-Sep-2026</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2391,12 +2391,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>01-Sep-2026</t>
+          <t>19-Sep-2026</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>EVER STEADY / 02633</t>
+          <t>ZHONG GU SHEN YANG / 02635</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2406,13 +2406,13 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>10 days</t>
+          <t>12 days</t>
         </is>
       </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2424,43 +2424,43 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>05-Sep-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>18-Sep-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>ZHONG GU SHEN YANG / 02635</t>
+          <t>ESL KABIR / 02638</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>13 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2472,12 +2472,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>14-Sep-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2487,28 +2487,28 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>ESL TBN1 / 02638</t>
+          <t>ESL NINGBO / 026E2</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>26-Sep-2026</t>
+          <t>25-Sep-2026</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2550,13 +2550,13 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>12 days</t>
+          <t>11 days</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14-Sep-2026</t>
+          <t>15-Sep-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2631,12 +2631,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>ESL NINGBO / 026E3</t>
+          <t>KMTC DAMMAM / 026E3</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2652,7 +2652,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>16-Sep-2026</t>
+          <t>18-Sep-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2679,12 +2679,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM / 026E1</t>
+          <t>ESL TBN01 / 026E4</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2700,7 +2700,7 @@
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>08-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2775,12 +2775,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>24-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>ESL TBN01 / 02640</t>
+          <t>KMT TBN / 02641</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2796,7 +2796,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2844,7 +2844,7 @@
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2856,12 +2856,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2871,28 +2871,28 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>24-Oct-2026</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>KMT TBN / 02641</t>
+          <t>BHUDTHI BHUM / 026E6</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2909,7 +2909,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>02-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2934,13 +2934,13 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>24 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -2957,38 +2957,42 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>03-Oct-2026</t>
+          <t>12-Aug-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM / 026E6</t>
+          <t>026D7</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>23 days</t>
-        </is>
-      </c>
-      <c r="I52" t="inlineStr"/>
+          <t>05-Sep-2026</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3005,38 +3009,42 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>16-Aug-2026</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
+          <t>ITAL USODIMARE</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>PHOEBE / 026E8</t>
+          <t>02632</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>23 days</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr"/>
+          <t>25-Aug-2026</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3048,47 +3056,47 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>09-Aug-2026</t>
+          <t>01-Sep-2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>EVER LIVING</t>
+          <t>ESL BUSAN</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>02630</t>
+          <t>02634</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>19-Aug-2026</t>
+          <t>12-Sep-2026</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3100,27 +3108,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>20-Aug-2026</t>
+          <t>21-Aug-2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ESL OMAN</t>
+          <t>PHOEBE</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>02633</t>
+          <t>026D9</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3130,17 +3138,17 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>05-Sep-2026</t>
+          <t>13-Sep-2026</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3157,42 +3165,42 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>12-Aug-2026</t>
+          <t>22-Aug-2026</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>EVER STEADY</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>026D7</t>
+          <t>02633</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>06-Sep-2026</t>
+          <t>01-Sep-2026</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>11</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3209,42 +3217,42 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>16-Aug-2026</t>
+          <t>28-Aug-2026</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>ITAL USODIMARE</t>
+          <t>ESL NHAVA SHEVA</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>02632</t>
+          <t>026E1</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>25-Aug-2026</t>
+          <t>20-Sep-2026</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3256,47 +3264,47 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
+          <t>QINGDAO</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>07-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ECSX</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>ZHONG GU SHEN YANG</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>02635</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
           <t>PORT KLANG</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>01-Sep-2026</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>EVGI</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>ESL BUSAN</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>02634</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>12-Sep-2026</t>
+          <t>19-Sep-2026</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3308,27 +3316,27 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>21-Aug-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>ESL KABIR</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>026D9</t>
+          <t>02638</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3338,17 +3346,17 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>13-Sep-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3365,42 +3373,42 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>22-Aug-2026</t>
+          <t>14-Sep-2026</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>EVER STEADY</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>02633</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>01-Sep-2026</t>
+          <t>07-Oct-2026</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3417,7 +3425,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>05-Sep-2026</t>
+          <t>14-Sep-2026</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3427,12 +3435,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>ZHONG GU SHEN YANG</t>
+          <t>TS SHANGHAI</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>02635</t>
+          <t>02637</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3442,17 +3450,17 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>18-Sep-2026</t>
+          <t>25-Sep-2026</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>12</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3469,7 +3477,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>24-Sep-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3479,12 +3487,12 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ESL TBN1</t>
+          <t>ESL OMAN</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>02638</t>
+          <t>02639</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3494,7 +3502,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>17-Oct-2026</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3504,7 +3512,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3521,42 +3529,42 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>14-Sep-2026</t>
+          <t>15-Sep-2026</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>TS SHANGHAI</t>
+          <t>KMTC DAMMAM</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>02637</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>26-Sep-2026</t>
+          <t>08-Oct-2026</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3568,27 +3576,27 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>18-Sep-2026</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>ESL OMAN</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>02639</t>
+          <t>026E4</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3598,17 +3606,17 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>17-Oct-2026</t>
+          <t>11-Oct-2026</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3625,42 +3633,42 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>14-Sep-2026</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ITAL USODIMARE</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>026E3</t>
+          <t>02638</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3672,27 +3680,27 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>16-Sep-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM</t>
+          <t>KMT TBN</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>026E1</t>
+          <t>02641</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3702,17 +3710,17 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>09-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3737,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>22-Sep-2026</t>
+          <t>28-Sep-2026</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3739,12 +3747,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>ITAL USODIMARE</t>
+          <t>EVER STEADY</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>02638</t>
+          <t>02639</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -3754,7 +3762,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>04-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
@@ -3764,7 +3772,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3776,27 +3784,27 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>08-Oct-2026</t>
+          <t>01-Oct-2026</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>ESL TBN01</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>02640</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3811,12 +3819,12 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3833,250 +3841,234 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>02-Oct-2026</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>EVER STEADY</t>
+          <t>ESL KHOR FAKKAN</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>02639</t>
+          <t>026E5</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>14-Aug-2026</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>KMT TBN</t>
+          <t>17-Aug-2026</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>02641</t>
+          <t>COSCO FOS / 00432</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
+          <t>3 days</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>18-Aug-2026</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>13-Sep-2026</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>PHOEBE / 026D9</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
           <t>EGLX</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>ESL KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr">
-        <is>
-          <t>026E5</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>25</t>
-        </is>
-      </c>
+          <t>26 days</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>XINGANG</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>03-Oct-2026</t>
+          <t>21-Aug-2026</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>24-Aug-2026</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>COSCO FOS / 00434</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>FCHS</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>26-Oct-2026</t>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
+          <t>3 days</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CNTAO→AEJEA</t>
+          <t>CNXNG→AEJEA</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>BUSAN</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16-Oct-2026</t>
+          <t>25-Aug-2026</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>ESL NHAVA SHEVA / 026E1</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
           <t>EGLX</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>PHOEBE</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>026E8</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>08-Nov-2026</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
+          <t>26 days</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4098,33 +4090,37 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>00432</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>17-Aug-2026</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>COSCO FOS / 00432</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4146,33 +4142,37 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
+          <t>PHOEBE</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>026D9</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>KHOR FAKKAN</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
           <t>13-Sep-2026</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>PHOEBE / 026D9</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>EGLX</t>
-        </is>
-      </c>
-      <c r="H75" t="inlineStr">
-        <is>
-          <t>26 days</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4194,33 +4194,37 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>COSCO FOS</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>00434</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
           <t>BUSAN</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>24-Aug-2026</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>COSCO FOS / 00434</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="H76" t="inlineStr">
-        <is>
-          <t>3 days</t>
-        </is>
-      </c>
-      <c r="I76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4237,246 +4241,234 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>11-Sep-2026</t>
+          <t>25-Aug-2026</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
+          <t>ESL NHAVA SHEVA</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>ESL NINGBO / 026E3</t>
+          <t>026E1</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>26 days</t>
-        </is>
-      </c>
-      <c r="I77" t="inlineStr"/>
+          <t>20-Sep-2026</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>14-Aug-2026</t>
+          <t>13-Aug-2026</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>21-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>FEEDER / 01059</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>COSCO FOS</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>00432</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>BUSAN</t>
-        </is>
-      </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>8 days</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>18-Aug-2026</t>
+          <t>25-Aug-2026</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>PHOEBE</t>
+          <t>12-Sep-2026</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>026D9</t>
+          <t>ESL SANA / 026D2</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>13-Sep-2026</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
+          <t>18 days</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>XINGANG</t>
+          <t>WUHAN</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>21-Aug-2026</t>
+          <t>17-Aug-2026</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
+          <t>SHANGHAI</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>25-Aug-2026</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>FEEDER / 01060</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
           <t>FCHS</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>COSCO FOS</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>00434</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>BUSAN</t>
-        </is>
-      </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>24-Aug-2026</t>
-        </is>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
+          <t>8 days</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CNXNG→AEJEA</t>
+          <t>CNWUH→AEJEA</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>BUSAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>11-Sep-2026</t>
+          <t>02-Sep-2026</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>22-Sep-2026</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>026E3</t>
+          <t>ESL TBN01 / 026D4</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>07-Oct-2026</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
+          <t>20 days</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr"/>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-08-13 01:56 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4493,7 +4485,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>09-Aug-2026</t>
+          <t>21-Aug-2026</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4503,12 +4495,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
+          <t>29-Aug-2026</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>FEEDER / 01058</t>
+          <t>FEEDER / 01061</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4524,7 +4516,7 @@
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr">
         <is>
-          <t>2026-08-13 01:57 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4536,43 +4528,47 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>13-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>01059</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>19-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>10-Sep-2026</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>KMTC COLOMBO / 026D1</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>22 days</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr"/>
+          <t>21-Aug-2026</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-08-13 01:57 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4584,43 +4580,47 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>13-Aug-2026</t>
+          <t>25-Aug-2026</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>21-Aug-2026</t>
+          <t>ESL SANA</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>FEEDER / 01059</t>
+          <t>026D2</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>8 days</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr"/>
+          <t>12-Sep-2026</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>2026-08-13 01:57 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4632,43 +4632,47 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>17-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>01060</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="H85" t="inlineStr">
         <is>
           <t>25-Aug-2026</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="E85" t="inlineStr">
-        <is>
-          <t>12-Sep-2026</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>ESL SANA / 026D2</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="H85" t="inlineStr">
-        <is>
-          <t>18 days</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>2026-08-13 01:57 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4680,43 +4684,47 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>WUHAN</t>
+          <t>SHANGHAI</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17-Aug-2026</t>
+          <t>02-Sep-2026</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>SHANGHAI</t>
+          <t>ECMX</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>25-Aug-2026</t>
+          <t>ESL TBN01</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>FEEDER / 01060</t>
+          <t>026D4</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>FCHS</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>8 days</t>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr"/>
+          <t>22-Sep-2026</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>2026-08-13 01:57 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4728,455 +4736,47 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
+          <t>WUHAN</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>21-Aug-2026</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>FCHS</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>FEEDER</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>01061</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
           <t>SHANGHAI</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>02-Sep-2026</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>22-Sep-2026</t>
-        </is>
-      </c>
-      <c r="F87" t="inlineStr">
-        <is>
-          <t>ESL NHAVA SHEVA / 026D4</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>20 days</t>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr"/>
+          <t>29-Aug-2026</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>21-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>29-Aug-2026</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>FEEDER / 01061</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="H88" t="inlineStr">
-        <is>
-          <t>8 days</t>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr"/>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>09-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>01058</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H89" t="inlineStr">
-        <is>
-          <t>17-Aug-2026</t>
-        </is>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>19-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr">
-        <is>
-          <t>KMTC COLOMBO</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr">
-        <is>
-          <t>026D1</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr">
-        <is>
-          <t>10-Sep-2026</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr">
-        <is>
-          <t>23</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>13-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr">
-        <is>
-          <t>01059</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr">
-        <is>
-          <t>21-Aug-2026</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>25-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr">
-        <is>
-          <t>ESL SANA</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr">
-        <is>
-          <t>026D2</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr">
-        <is>
-          <t>12-Sep-2026</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>17-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>01060</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr">
-        <is>
-          <t>25-Aug-2026</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>02-Sep-2026</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>ECMX</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>ESL NHAVA SHEVA</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>026D4</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr">
-        <is>
-          <t>22-Sep-2026</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
-        <is>
-          <t>CNWUH→AEJEA</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>WUHAN</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr">
-        <is>
-          <t>21-Aug-2026</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>FCHS</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>FEEDER</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>01061</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>SHANGHAI</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr">
-        <is>
-          <t>29-Aug-2026</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>2026-08-13 01:57 UTC</t>
+          <t>2026-08-14 01:54 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>